<commit_message>
fix: change the mediate to prediction
</commit_message>
<xml_diff>
--- a/tables/country_level_effect_summary.xlsx
+++ b/tables/country_level_effect_summary.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.0209</t>
+          <t>0.0208</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -522,22 +522,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>(0.0006)</t>
+          <t>(0.0086)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>(0.0002)</t>
+          <t>(0.0090)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>(0.0098)</t>
+          <t>(0.0045)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>(0.0100)</t>
+          <t>(0.0048)</t>
         </is>
       </c>
     </row>
@@ -554,22 +554,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.0113</t>
+          <t>0.0105</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-0.0005</t>
+          <t>-0.0013</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.2384</t>
+          <t>0.2375</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.2243</t>
+          <t>0.2235</t>
         </is>
       </c>
     </row>
@@ -582,22 +582,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>(0.0006)</t>
+          <t>(0.0119)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>(0.0003)</t>
+          <t>(0.0118)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>(0.0135)</t>
+          <t>(0.0076)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>(0.0133)</t>
+          <t>(0.0074)</t>
         </is>
       </c>
     </row>
@@ -614,22 +614,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.0048</t>
+          <t>0.0060</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-0.0011</t>
+          <t>0.0001</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.2932</t>
+          <t>0.2944</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.2821</t>
+          <t>0.2833</t>
         </is>
       </c>
     </row>
@@ -642,22 +642,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>(0.0006)</t>
+          <t>(0.0067)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>(0.0004)</t>
+          <t>(0.0068)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>(0.0075)</t>
+          <t>(0.0040)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>(0.0074)</t>
+          <t>(0.0040)</t>
         </is>
       </c>
     </row>
@@ -674,22 +674,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.0717</t>
+          <t>0.0770</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-0.0030</t>
+          <t>0.0023</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.8705</t>
+          <t>0.8758</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0.8440</t>
+          <t>0.8493</t>
         </is>
       </c>
     </row>
@@ -702,22 +702,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>(0.0013)</t>
+          <t>(0.0101)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>(0.0006)</t>
+          <t>(0.0108)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>(0.0111)</t>
+          <t>(0.0067)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>(0.0112)</t>
+          <t>(0.0063)</t>
         </is>
       </c>
     </row>
@@ -734,22 +734,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>-0.0162</t>
+          <t>-0.0094</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.0022</t>
+          <t>0.0091</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.5820</t>
+          <t>0.5889</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0.5983</t>
+          <t>0.6051</t>
         </is>
       </c>
     </row>
@@ -762,22 +762,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>(0.0003)</t>
+          <t>(0.0079)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>(0.0001)</t>
+          <t>(0.0080)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>(0.0095)</t>
+          <t>(0.0052)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>(0.0093)</t>
+          <t>(0.0052)</t>
         </is>
       </c>
     </row>
@@ -794,22 +794,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.0566</t>
+          <t>0.0535</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-0.0042</t>
+          <t>-0.0073</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.5608</t>
+          <t>0.5577</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.5060</t>
+          <t>0.5028</t>
         </is>
       </c>
     </row>
@@ -822,22 +822,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>(0.0018)</t>
+          <t>(0.0064)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>(0.0005)</t>
+          <t>(0.0061)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>(0.0068)</t>
+          <t>(0.0039)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>(0.0066)</t>
+          <t>(0.0037)</t>
         </is>
       </c>
     </row>
@@ -854,22 +854,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>-0.0410</t>
+          <t>-0.0370</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>-0.0030</t>
+          <t>0.0011</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0.1163</t>
+          <t>0.1203</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.1529</t>
+          <t>0.1569</t>
         </is>
       </c>
     </row>
@@ -882,22 +882,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>(0.0013)</t>
+          <t>(0.0050)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>(0.0005)</t>
+          <t>(0.0050)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>(0.0052)</t>
+          <t>(0.0025)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>(0.0051)</t>
+          <t>(0.0024)</t>
         </is>
       </c>
     </row>
@@ -914,22 +914,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>-0.1044</t>
+          <t>-0.1112</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.0081</t>
+          <t>-0.0150</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0.1483</t>
+          <t>0.1415</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0.2661</t>
+          <t>0.2593</t>
         </is>
       </c>
     </row>
@@ -942,22 +942,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>(0.0012)</t>
+          <t>(0.0098)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>(0.0007)</t>
+          <t>(0.0099)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>(0.0111)</t>
+          <t>(0.0065)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>(0.0114)</t>
+          <t>(0.0066)</t>
         </is>
       </c>
     </row>
@@ -974,22 +974,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.0121</t>
+          <t>0.0114</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>-0.0008</t>
+          <t>-0.0015</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0.4049</t>
+          <t>0.4042</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0.3948</t>
+          <t>0.3941</t>
         </is>
       </c>
     </row>
@@ -1002,22 +1002,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>(0.0002)</t>
+          <t>(0.0046)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>(0.0002)</t>
+          <t>(0.0047)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>(0.0047)</t>
+          <t>(0.0023)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>(0.0049)</t>
+          <t>(0.0023)</t>
         </is>
       </c>
     </row>
@@ -1034,22 +1034,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>-0.0054</t>
+          <t>0.0002</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>-0.0094</t>
+          <t>-0.0038</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>0.3679</t>
+          <t>0.3735</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0.3636</t>
+          <t>0.3692</t>
         </is>
       </c>
     </row>
@@ -1062,22 +1062,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>(0.0007)</t>
+          <t>(0.0043)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>(0.0005)</t>
+          <t>(0.0044)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>(0.0048)</t>
+          <t>(0.0028)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>(0.0049)</t>
+          <t>(0.0028)</t>
         </is>
       </c>
     </row>
@@ -1094,22 +1094,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-0.0057</t>
+          <t>-0.0029</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-0.0014</t>
+          <t>0.0014</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0.2398</t>
+          <t>0.2426</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0.2399</t>
+          <t>0.2426</t>
         </is>
       </c>
     </row>
@@ -1122,22 +1122,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>(0.0006)</t>
+          <t>(0.0078)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>(0.0004)</t>
+          <t>(0.0078)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>(0.0086)</t>
+          <t>(0.0043)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>(0.0090)</t>
+          <t>(0.0041)</t>
         </is>
       </c>
     </row>
@@ -1154,22 +1154,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>-0.0250</t>
+          <t>-0.0216</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.0017</t>
+          <t>0.0051</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0.2932</t>
+          <t>0.2965</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>0.3095</t>
+          <t>0.3129</t>
         </is>
       </c>
     </row>
@@ -1182,22 +1182,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>(0.0013)</t>
+          <t>(0.0054)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>(0.0005)</t>
+          <t>(0.0053)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>(0.0055)</t>
+          <t>(0.0026)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>(0.0055)</t>
+          <t>(0.0026)</t>
         </is>
       </c>
     </row>
@@ -1214,22 +1214,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>-0.0263</t>
+          <t>-0.0298</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0.0016</t>
+          <t>-0.0020</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0.2001</t>
+          <t>0.1965</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0.2337</t>
+          <t>0.2302</t>
         </is>
       </c>
     </row>
@@ -1242,22 +1242,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>(0.0014)</t>
+          <t>(0.0052)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>(0.0006)</t>
+          <t>(0.0052)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>(0.0052)</t>
+          <t>(0.0032)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>(0.0053)</t>
+          <t>(0.0029)</t>
         </is>
       </c>
     </row>
@@ -1274,22 +1274,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>-0.0160</t>
+          <t>-0.0166</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0.0011</t>
+          <t>0.0004</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>0.2580</t>
+          <t>0.2574</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0.2891</t>
+          <t>0.2885</t>
         </is>
       </c>
     </row>
@@ -1302,22 +1302,22 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>(0.0006)</t>
+          <t>(0.0047)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>(0.0003)</t>
+          <t>(0.0046)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>(0.0053)</t>
+          <t>(0.0037)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>(0.0054)</t>
+          <t>(0.0034)</t>
         </is>
       </c>
     </row>
@@ -1334,22 +1334,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.0070</t>
+          <t>0.0024</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>-0.0004</t>
+          <t>-0.0050</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>0.3612</t>
+          <t>0.3566</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>0.3503</t>
+          <t>0.3457</t>
         </is>
       </c>
     </row>
@@ -1362,22 +1362,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>(0.0014)</t>
+          <t>(0.0130)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>(0.0005)</t>
+          <t>(0.0130)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>(0.0128)</t>
+          <t>(0.0070)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>(0.0132)</t>
+          <t>(0.0072)</t>
         </is>
       </c>
     </row>
@@ -1394,22 +1394,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.0171</t>
+          <t>0.0127</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>-0.0005</t>
+          <t>-0.0049</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0.3314</t>
+          <t>0.3270</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>0.3151</t>
+          <t>0.3107</t>
         </is>
       </c>
     </row>
@@ -1422,22 +1422,22 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>(0.0004)</t>
+          <t>(0.0094)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>(0.0002)</t>
+          <t>(0.0096)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>(0.0106)</t>
+          <t>(0.0051)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>(0.0107)</t>
+          <t>(0.0050)</t>
         </is>
       </c>
     </row>
@@ -1454,22 +1454,22 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>-0.0432</t>
+          <t>-0.0450</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>-0.0177</t>
+          <t>-0.0195</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>0.3469</t>
+          <t>0.3451</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>0.3704</t>
+          <t>0.3687</t>
         </is>
       </c>
     </row>
@@ -1482,22 +1482,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>(0.0010)</t>
+          <t>(0.0060)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>(0.0009)</t>
+          <t>(0.0060)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>(0.0066)</t>
+          <t>(0.0043)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>(0.0066)</t>
+          <t>(0.0042)</t>
         </is>
       </c>
     </row>
@@ -1514,22 +1514,22 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.0166</t>
+          <t>0.0435</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>-0.0002</t>
+          <t>0.0267</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>0.4248</t>
+          <t>0.4517</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>0.4092</t>
+          <t>0.4361</t>
         </is>
       </c>
     </row>
@@ -1542,22 +1542,22 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>(0.0010)</t>
+          <t>(0.0190)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>(0.0005)</t>
+          <t>(0.0200)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>(0.0209)</t>
+          <t>(0.0101)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>(0.0203)</t>
+          <t>(0.0096)</t>
         </is>
       </c>
     </row>
@@ -1574,22 +1574,22 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>-0.0219</t>
+          <t>-0.0225</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>0.0038</t>
+          <t>0.0032</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>0.5647</t>
+          <t>0.5641</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>0.5866</t>
+          <t>0.5860</t>
         </is>
       </c>
     </row>
@@ -1602,22 +1602,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>(0.0005)</t>
+          <t>(0.0117)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>(0.0002)</t>
+          <t>(0.0120)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>(0.0148)</t>
+          <t>(0.0081)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>(0.0144)</t>
+          <t>(0.0084)</t>
         </is>
       </c>
     </row>
@@ -1634,22 +1634,22 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.0013</t>
+          <t>0.0017</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>0.0003</t>
+          <t>0.0008</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>0.2956</t>
+          <t>0.2960</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>0.2933</t>
+          <t>0.2938</t>
         </is>
       </c>
     </row>
@@ -1662,22 +1662,22 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>(0.0001)</t>
+          <t>(0.0038)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>(0.0000)</t>
+          <t>(0.0037)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>(0.0041)</t>
+          <t>(0.0021)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>(0.0043)</t>
+          <t>(0.0021)</t>
         </is>
       </c>
     </row>
@@ -1694,22 +1694,22 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.0228</t>
+          <t>0.0218</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>-0.0037</t>
+          <t>-0.0047</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>-0.0209</t>
+          <t>-0.0219</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>-0.0685</t>
+          <t>-0.0696</t>
         </is>
       </c>
     </row>
@@ -1722,22 +1722,22 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>(0.0003)</t>
+          <t>(0.0059)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>(0.0002)</t>
+          <t>(0.0062)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>(0.0073)</t>
+          <t>(0.0036)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>(0.0071)</t>
+          <t>(0.0037)</t>
         </is>
       </c>
     </row>
@@ -1754,22 +1754,22 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>-0.1248</t>
+          <t>-0.1190</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>0.0050</t>
+          <t>0.0108</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>-0.3631</t>
+          <t>-0.3573</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>-0.2217</t>
+          <t>-0.2159</t>
         </is>
       </c>
     </row>
@@ -1782,22 +1782,22 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>(0.0028)</t>
+          <t>(0.0079)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>(0.0012)</t>
+          <t>(0.0076)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>(0.0095)</t>
+          <t>(0.0076)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>(0.0091)</t>
+          <t>(0.0071)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: revise the mediate effect
</commit_message>
<xml_diff>
--- a/tables/country_level_effect_summary.xlsx
+++ b/tables/country_level_effect_summary.xlsx
@@ -494,12 +494,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.0208</t>
+          <t>0.0215</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>-0.0028</t>
+          <t>-0.0022</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -522,22 +522,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>(0.0086)</t>
+          <t>(0.0005)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>(0.0090)</t>
+          <t>(0.0002)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>(0.0045)</t>
+          <t>(0.0047)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>(0.0048)</t>
+          <t>(0.0047)</t>
         </is>
       </c>
     </row>
@@ -554,12 +554,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.0105</t>
+          <t>0.0064</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-0.0013</t>
+          <t>-0.0011</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -582,12 +582,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>(0.0119)</t>
+          <t>(0.0005)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>(0.0118)</t>
+          <t>(0.0002)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>(0.0074)</t>
+          <t>(0.0071)</t>
         </is>
       </c>
     </row>
@@ -614,12 +614,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.0060</t>
+          <t>0.0040</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.0001</t>
+          <t>-0.0018</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -642,17 +642,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>(0.0067)</t>
+          <t>(0.0005)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>(0.0068)</t>
+          <t>(0.0003)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>(0.0040)</t>
+          <t>(0.0039)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -674,12 +674,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.0770</t>
+          <t>0.0529</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.0023</t>
+          <t>-0.0004</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -702,17 +702,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>(0.0101)</t>
+          <t>(0.0010)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>(0.0108)</t>
+          <t>(0.0005)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>(0.0067)</t>
+          <t>(0.0064)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -734,12 +734,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>-0.0094</t>
+          <t>-0.0116</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.0091</t>
+          <t>0.0003</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -762,22 +762,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>(0.0079)</t>
+          <t>(0.0002)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>(0.0080)</t>
+          <t>(0.0001)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>(0.0052)</t>
+          <t>(0.0051)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>(0.0052)</t>
+          <t>(0.0054)</t>
         </is>
       </c>
     </row>
@@ -794,12 +794,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.0535</t>
+          <t>0.0490</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-0.0073</t>
+          <t>-0.0042</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -822,22 +822,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>(0.0064)</t>
+          <t>(0.0014)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>(0.0061)</t>
+          <t>(0.0004)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>(0.0039)</t>
+          <t>(0.0040)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>(0.0037)</t>
+          <t>(0.0040)</t>
         </is>
       </c>
     </row>
@@ -854,12 +854,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>-0.0370</t>
+          <t>-0.0344</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.0011</t>
+          <t>-0.0004</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -882,22 +882,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>(0.0050)</t>
+          <t>(0.0010)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>(0.0050)</t>
+          <t>(0.0003)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>(0.0025)</t>
+          <t>(0.0026)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>(0.0024)</t>
+          <t>(0.0022)</t>
         </is>
       </c>
     </row>
@@ -914,12 +914,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>-0.1112</t>
+          <t>-0.0594</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.0150</t>
+          <t>0.0002</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -942,22 +942,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>(0.0098)</t>
+          <t>(0.0012)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>(0.0099)</t>
+          <t>(0.0004)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
+          <t>(0.0066)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
           <t>(0.0065)</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>(0.0066)</t>
         </is>
       </c>
     </row>
@@ -974,12 +974,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.0114</t>
+          <t>0.0103</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>-0.0015</t>
+          <t>-0.0030</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1002,12 +1002,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>(0.0046)</t>
+          <t>(0.0002)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>(0.0047)</t>
+          <t>(0.0001)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1034,12 +1034,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.0002</t>
+          <t>-0.0032</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>-0.0038</t>
+          <t>-0.0101</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1062,12 +1062,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>(0.0043)</t>
+          <t>(0.0005)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>(0.0044)</t>
+          <t>(0.0004)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1077,7 +1077,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>(0.0028)</t>
+          <t>(0.0027)</t>
         </is>
       </c>
     </row>
@@ -1094,12 +1094,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>-0.0029</t>
+          <t>-0.0002</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.0014</t>
+          <t>-0.0008</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1122,22 +1122,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>(0.0078)</t>
+          <t>(0.0006)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>(0.0078)</t>
+          <t>(0.0002)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>(0.0043)</t>
+          <t>(0.0042)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>(0.0041)</t>
+          <t>(0.0042)</t>
         </is>
       </c>
     </row>
@@ -1154,12 +1154,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>-0.0216</t>
+          <t>-0.0116</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.0051</t>
+          <t>0.0003</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1182,22 +1182,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>(0.0054)</t>
+          <t>(0.0009)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>(0.0053)</t>
+          <t>(0.0003)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>(0.0026)</t>
+          <t>(0.0027)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>(0.0026)</t>
+          <t>(0.0025)</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>-0.0298</t>
+          <t>-0.0196</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>-0.0020</t>
+          <t>0.0004</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1242,22 +1242,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>(0.0052)</t>
+          <t>(0.0013)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>(0.0052)</t>
+          <t>(0.0004)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>(0.0032)</t>
+          <t>(0.0033)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>(0.0029)</t>
+          <t>(0.0028)</t>
         </is>
       </c>
     </row>
@@ -1274,12 +1274,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>-0.0166</t>
+          <t>0.0069</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0.0004</t>
+          <t>-0.0024</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1302,22 +1302,22 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>(0.0047)</t>
+          <t>(0.0006)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>(0.0046)</t>
+          <t>(0.0003)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>(0.0037)</t>
+          <t>(0.0035)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>(0.0034)</t>
+          <t>(0.0036)</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1334,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>0.0024</t>
+          <t>0.0124</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>-0.0050</t>
+          <t>-0.0008</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1362,22 +1362,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>(0.0130)</t>
+          <t>(0.0009)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>(0.0130)</t>
+          <t>(0.0004)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>(0.0070)</t>
+          <t>(0.0071)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>(0.0072)</t>
+          <t>(0.0069)</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1394,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.0127</t>
+          <t>0.0129</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>-0.0049</t>
+          <t>-0.0001</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1422,17 +1422,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>(0.0094)</t>
+          <t>(0.0003)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>(0.0096)</t>
+          <t>(0.0001)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>(0.0051)</t>
+          <t>(0.0049)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1454,12 +1454,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>-0.0450</t>
+          <t>-0.0379</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>-0.0195</t>
+          <t>-0.0157</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1482,22 +1482,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>(0.0060)</t>
+          <t>(0.0008)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>(0.0060)</t>
+          <t>(0.0006)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>(0.0043)</t>
+          <t>(0.0042)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>(0.0042)</t>
+          <t>(0.0041)</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0.0435</t>
+          <t>0.0150</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>0.0267</t>
+          <t>-0.0012</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1542,22 +1542,22 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>(0.0190)</t>
+          <t>(0.0008)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>(0.0200)</t>
+          <t>(0.0003)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>(0.0101)</t>
+          <t>(0.0100)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>(0.0096)</t>
+          <t>(0.0100)</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>-0.0225</t>
+          <t>-0.0226</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>0.0032</t>
+          <t>0.0021</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1602,22 +1602,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>(0.0117)</t>
+          <t>(0.0005)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>(0.0120)</t>
+          <t>(0.0002)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>(0.0081)</t>
+          <t>(0.0082)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>(0.0084)</t>
+          <t>(0.0079)</t>
         </is>
       </c>
     </row>
@@ -1634,12 +1634,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0.0017</t>
+          <t>0.0021</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>0.0008</t>
+          <t>0.0004</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1662,17 +1662,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>(0.0038)</t>
+          <t>(0.0001)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>(0.0037)</t>
+          <t>(0.0000)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>(0.0021)</t>
+          <t>(0.0022)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -1694,12 +1694,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0.0218</t>
+          <t>0.0186</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>-0.0047</t>
+          <t>-0.0018</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1722,22 +1722,22 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>(0.0059)</t>
+          <t>(0.0002)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>(0.0062)</t>
+          <t>(0.0001)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>(0.0036)</t>
+          <t>(0.0039)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>(0.0037)</t>
+          <t>(0.0039)</t>
         </is>
       </c>
     </row>
@@ -1754,12 +1754,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>-0.1190</t>
+          <t>-0.1001</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>0.0108</t>
+          <t>0.0012</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1782,12 +1782,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>(0.0079)</t>
+          <t>(0.0020)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>(0.0076)</t>
+          <t>(0.0008)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">

</xml_diff>